<commit_message>
Compress Arrow of Light: all six required adventures done by Feb 11 before crossover (Outdoor Adventurer to Nov campout; Feb doubles up)
</commit_message>
<xml_diff>
--- a/downloads/Pack 925 - Den Planning Grid.xlsx
+++ b/downloads/Pack 925 - Den Planning Grid.xlsx
@@ -969,7 +969,7 @@
       </c>
       <c r="G6" s="13" t="inlineStr">
         <is>
-          <t>Personal Fitness</t>
+          <t>Outdoor Adventurer</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>Citizenship</t>
+          <t>Personal Fitness</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="G8" s="13" t="inlineStr">
         <is>
-          <t>Duty to God</t>
+          <t>Citizenship &amp; Duty to God</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>Outdoor Adventurer</t>
+          <t>Complete - Optional: Knife Safety</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>Knife Safety (elective) + Catch-Up</t>
+          <t>Crossed Over - Mentor &amp; Celebrate</t>
         </is>
       </c>
     </row>
@@ -4412,7 +4412,7 @@
       </c>
       <c r="C76" s="13" t="inlineStr">
         <is>
-          <t>Personal Fitness</t>
+          <t>Outdoor Adventurer</t>
         </is>
       </c>
       <c r="D76" s="13" t="inlineStr">
@@ -4422,268 +4422,10 @@
       </c>
       <c r="E76" s="13" t="inlineStr">
         <is>
-          <t>Camp Meal Plan and Cook</t>
+          <t>Campout Prep and Patrol Plan</t>
         </is>
       </c>
       <c r="F76" s="13" t="inlineStr">
-        <is>
-          <t>Personal Fitness 1 (Plan a balanced meal for camping; prepare it using camp gear)</t>
-        </is>
-      </c>
-      <c r="G76" s="13" t="inlineStr">
-        <is>
-          <t>menu planning sheets, pencils, sample camp gear list, camp stove or backpacking stove, fuel handled by adults, cook pot or skillet, utensils, wash station, meal ingredients</t>
-        </is>
-      </c>
-      <c r="H76" s="13" t="inlineStr">
-        <is>
-          <t>Start or continue the 14-day activity tracker.
-Ask parents to review the BSA Annual Health and Medical Record with you.</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="14" t="inlineStr">
-        <is>
-          <t>Arrow of Light</t>
-        </is>
-      </c>
-      <c r="B77" s="13" t="inlineStr">
-        <is>
-          <t>November 2026</t>
-        </is>
-      </c>
-      <c r="C77" s="13" t="inlineStr">
-        <is>
-          <t>Personal Fitness</t>
-        </is>
-      </c>
-      <c r="D77" s="13" t="inlineStr">
-        <is>
-          <t>Thu Nov 19</t>
-        </is>
-      </c>
-      <c r="E77" s="13" t="inlineStr">
-        <is>
-          <t>Patrol Fitness Challenge</t>
-        </is>
-      </c>
-      <c r="F77" s="13" t="inlineStr">
-        <is>
-          <t>Personal Fitness 2 (Share 14-day activity tracking - if completed)
-Personal Fitness 3 (Active 30 minutes with patrol/another person including stretching and moving)</t>
-        </is>
-      </c>
-      <c r="G77" s="13" t="inlineStr">
-        <is>
-          <t>open space, cones, stopwatch, water access, activity trackers, pencils</t>
-        </is>
-      </c>
-      <c r="H77" s="13" t="inlineStr">
-        <is>
-          <t>Finish the 14-day tracker if needed and share it with the den leader.
-Confirm the health record review is complete.</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="14" t="inlineStr">
-        <is>
-          <t>Arrow of Light</t>
-        </is>
-      </c>
-      <c r="B78" s="13" t="inlineStr">
-        <is>
-          <t>January 2027</t>
-        </is>
-      </c>
-      <c r="C78" s="13" t="inlineStr">
-        <is>
-          <t>Citizenship</t>
-        </is>
-      </c>
-      <c r="D78" s="13" t="inlineStr">
-        <is>
-          <t>Thu Jan 7</t>
-        </is>
-      </c>
-      <c r="E78" s="13" t="inlineStr">
-        <is>
-          <t>Choose and Plan Service</t>
-        </is>
-      </c>
-      <c r="F78" s="13" t="inlineStr">
-        <is>
-          <t>Citizenship 1 (Identify a service project and use the BSA SAFE Checklist to plan it safely)</t>
-        </is>
-      </c>
-      <c r="G78" s="13" t="inlineStr">
-        <is>
-          <t>project idea list, pencils, planning worksheet, BSA SAFE Checklist copy, chart paper, markers</t>
-        </is>
-      </c>
-      <c r="H78" s="13" t="inlineStr">
-        <is>
-          <t>Share the service date, location, clothing, and permission needs with families.
-Ask families to protect a full two-hour service block or plan make-up service.</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="14" t="inlineStr">
-        <is>
-          <t>Arrow of Light</t>
-        </is>
-      </c>
-      <c r="B79" s="13" t="inlineStr">
-        <is>
-          <t>January 2027</t>
-        </is>
-      </c>
-      <c r="C79" s="13" t="inlineStr">
-        <is>
-          <t>Citizenship</t>
-        </is>
-      </c>
-      <c r="D79" s="13" t="inlineStr">
-        <is>
-          <t>Thu Jan 21</t>
-        </is>
-      </c>
-      <c r="E79" s="13" t="inlineStr">
-        <is>
-          <t>Service Project Work Session</t>
-        </is>
-      </c>
-      <c r="F79" s="13" t="inlineStr">
-        <is>
-          <t>Citizenship 2 (Participate in a service project for at least two hours total - complete during project/outing if time requirement is met)</t>
-        </is>
-      </c>
-      <c r="G79" s="13" t="inlineStr">
-        <is>
-          <t>project-specific supplies, work gloves, trash bags or boxes, first-aid kit, water, service hour log, pencils</t>
-        </is>
-      </c>
-      <c r="H79" s="13" t="inlineStr">
-        <is>
-          <t>If you did not reach two service hours, finish approved make-up service before April advancement closeout.</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="14" t="inlineStr">
-        <is>
-          <t>Arrow of Light</t>
-        </is>
-      </c>
-      <c r="B80" s="13" t="inlineStr">
-        <is>
-          <t>February 2027</t>
-        </is>
-      </c>
-      <c r="C80" s="13" t="inlineStr">
-        <is>
-          <t>Duty to God</t>
-        </is>
-      </c>
-      <c r="D80" s="13" t="inlineStr">
-        <is>
-          <t>Thu Feb 4</t>
-        </is>
-      </c>
-      <c r="E80" s="13" t="inlineStr">
-        <is>
-          <t>Values and Crisis Helpers</t>
-        </is>
-      </c>
-      <c r="F80" s="13" t="inlineStr">
-        <is>
-          <t>Duty to God 2 (Meet with a representative of a faith-based organization that assists people in crisis regardless of faith - if guest attends tonight)</t>
-        </is>
-      </c>
-      <c r="G80" s="13" t="inlineStr">
-        <is>
-          <t>index cards, pencils, guest/visit confirmation, thank-you card, question cards</t>
-        </is>
-      </c>
-      <c r="H80" s="13" t="inlineStr">
-        <is>
-          <t>Complete the family faith/value discussion (req 1).
-Start thinking about how you practice Duty to God daily (req 3).</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="14" t="inlineStr">
-        <is>
-          <t>Arrow of Light</t>
-        </is>
-      </c>
-      <c r="B81" s="13" t="inlineStr">
-        <is>
-          <t>February 2027</t>
-        </is>
-      </c>
-      <c r="C81" s="13" t="inlineStr">
-        <is>
-          <t>Duty to God</t>
-        </is>
-      </c>
-      <c r="D81" s="13" t="inlineStr">
-        <is>
-          <t>Thu Feb 11</t>
-        </is>
-      </c>
-      <c r="E81" s="13" t="inlineStr">
-        <is>
-          <t>Duty in Daily Life</t>
-        </is>
-      </c>
-      <c r="F81" s="13" t="inlineStr">
-        <is>
-          <t>Duty to God 2 (Crisis-helping organization discussion/visit wrap-up)
-Duty to God 3 (Discuss what Duty to God means and daily practice - if done with adult leader tonight)</t>
-        </is>
-      </c>
-      <c r="G81" s="13" t="inlineStr">
-        <is>
-          <t>notes from visit/guest, thank-you card, markers</t>
-        </is>
-      </c>
-      <c r="H81" s="13" t="inlineStr">
-        <is>
-          <t>Finish any remaining Duty to God home discussions with a parent/guardian.</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="14" t="inlineStr">
-        <is>
-          <t>Arrow of Light</t>
-        </is>
-      </c>
-      <c r="B82" s="13" t="inlineStr">
-        <is>
-          <t>March 2027</t>
-        </is>
-      </c>
-      <c r="C82" s="13" t="inlineStr">
-        <is>
-          <t>Outdoor Adventurer</t>
-        </is>
-      </c>
-      <c r="D82" s="13" t="inlineStr">
-        <is>
-          <t>Thu Mar 4</t>
-        </is>
-      </c>
-      <c r="E82" s="13" t="inlineStr">
-        <is>
-          <t>Campout Prep and Patrol Plan</t>
-        </is>
-      </c>
-      <c r="F82" s="13" t="inlineStr">
         <is>
           <t>Outdoor Adventurer 1 (Scout Basic Essentials)
 Outdoor Adventurer 2 (What to bring and how to carry it)
@@ -4691,15 +4433,279 @@
 Outdoor Adventurer 4 (Locate camp and campsite on a map)</t>
         </is>
       </c>
+      <c r="G76" s="13" t="inlineStr">
+        <is>
+          <t>packing checklist, pencils, sample gear, BSA SAFE Checklist, chart paper, markers, camp map, printed site map or blank paper</t>
+        </is>
+      </c>
+      <c r="H76" s="13" t="inlineStr">
+        <is>
+          <t>Start gathering cold-weather layers and sleeping gear for Nov 20-22.
+Turn in any required medical forms/permission for the campout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="14" t="inlineStr">
+        <is>
+          <t>Arrow of Light</t>
+        </is>
+      </c>
+      <c r="B77" s="13" t="inlineStr">
+        <is>
+          <t>November 2026</t>
+        </is>
+      </c>
+      <c r="C77" s="13" t="inlineStr">
+        <is>
+          <t>Outdoor Adventurer</t>
+        </is>
+      </c>
+      <c r="D77" s="13" t="inlineStr">
+        <is>
+          <t>Thu Nov 19</t>
+        </is>
+      </c>
+      <c r="E77" s="13" t="inlineStr">
+        <is>
+          <t>Final Prep: Camp Kitchen &amp; Setup Skills</t>
+        </is>
+      </c>
+      <c r="F77" s="13" t="inlineStr">
+        <is>
+          <t>Outdoor Adventurer 6 prep (Campsite setup and patrol-gear-first plan - demonstrated at the campout)
+Outdoor Adventurer 7 prep (Food safety and kitchen sanitation - demonstrated at the campout)</t>
+        </is>
+      </c>
+      <c r="G77" s="13" t="inlineStr">
+        <is>
+          <t>a tent or two, ground cloth, cones or rope to mark areas, 3 wash bins, biodegradable soap, sanitizer, dish towels, food storage bins</t>
+        </is>
+      </c>
+      <c r="H77" s="13" t="inlineStr">
+        <is>
+          <t>Finish packing for Nov 20-22 using your checklist.
+At the campout: set patrol gear first, keep the kitchen sanitary, and join the Sunday-morning debrief to finish the adventure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="14" t="inlineStr">
+        <is>
+          <t>Arrow of Light</t>
+        </is>
+      </c>
+      <c r="B78" s="13" t="inlineStr">
+        <is>
+          <t>January 2027</t>
+        </is>
+      </c>
+      <c r="C78" s="13" t="inlineStr">
+        <is>
+          <t>Personal Fitness</t>
+        </is>
+      </c>
+      <c r="D78" s="13" t="inlineStr">
+        <is>
+          <t>Thu Jan 7</t>
+        </is>
+      </c>
+      <c r="E78" s="13" t="inlineStr">
+        <is>
+          <t>Camp Meal Plan and Cook</t>
+        </is>
+      </c>
+      <c r="F78" s="13" t="inlineStr">
+        <is>
+          <t>Personal Fitness 1 (Plan a balanced meal for camping; prepare it using camp gear)</t>
+        </is>
+      </c>
+      <c r="G78" s="13" t="inlineStr">
+        <is>
+          <t>menu planning sheets, pencils, sample camp gear list, camp stove or backpacking stove, fuel handled by adults, cook pot or skillet, utensils, wash station, meal ingredients</t>
+        </is>
+      </c>
+      <c r="H78" s="13" t="inlineStr">
+        <is>
+          <t>Start or continue the 14-day activity tracker.
+Ask parents to review the BSA Annual Health and Medical Record with you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="14" t="inlineStr">
+        <is>
+          <t>Arrow of Light</t>
+        </is>
+      </c>
+      <c r="B79" s="13" t="inlineStr">
+        <is>
+          <t>January 2027</t>
+        </is>
+      </c>
+      <c r="C79" s="13" t="inlineStr">
+        <is>
+          <t>Personal Fitness</t>
+        </is>
+      </c>
+      <c r="D79" s="13" t="inlineStr">
+        <is>
+          <t>Thu Jan 21</t>
+        </is>
+      </c>
+      <c r="E79" s="13" t="inlineStr">
+        <is>
+          <t>Patrol Fitness Challenge</t>
+        </is>
+      </c>
+      <c r="F79" s="13" t="inlineStr">
+        <is>
+          <t>Personal Fitness 2 (Share 14-day activity tracking - if completed)
+Personal Fitness 3 (Active 30 minutes with patrol/another person including stretching and moving)</t>
+        </is>
+      </c>
+      <c r="G79" s="13" t="inlineStr">
+        <is>
+          <t>open space, cones, stopwatch, water access, activity trackers, pencils</t>
+        </is>
+      </c>
+      <c r="H79" s="13" t="inlineStr">
+        <is>
+          <t>Finish the 14-day tracker if needed and share it with the den leader.
+Confirm the health record review is complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="14" t="inlineStr">
+        <is>
+          <t>Arrow of Light</t>
+        </is>
+      </c>
+      <c r="B80" s="13" t="inlineStr">
+        <is>
+          <t>February 2027</t>
+        </is>
+      </c>
+      <c r="C80" s="13" t="inlineStr">
+        <is>
+          <t>Citizenship &amp; Duty to God</t>
+        </is>
+      </c>
+      <c r="D80" s="13" t="inlineStr">
+        <is>
+          <t>Thu Feb 4</t>
+        </is>
+      </c>
+      <c r="E80" s="13" t="inlineStr">
+        <is>
+          <t>Citizenship: Plan &amp; Serve</t>
+        </is>
+      </c>
+      <c r="F80" s="13" t="inlineStr">
+        <is>
+          <t>Citizenship 1 (Identify a service project and use the BSA SAFE Checklist to plan it safely)
+Citizenship 2 (Two hours of service total - completed at Scouting for Food Feb 6 &amp; 13 or another approved project)</t>
+        </is>
+      </c>
+      <c r="G80" s="13" t="inlineStr">
+        <is>
+          <t>BSA SAFE Checklist copy, project idea list, planning worksheet, pencils, service hour log, work gloves, collection bags or boxes</t>
+        </is>
+      </c>
+      <c r="H80" s="13" t="inlineStr">
+        <is>
+          <t>Protect the Scouting for Food dates (Feb 6 &amp; 13) so everyone reaches two service hours.
+Log service hours in Scoutbook right away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="14" t="inlineStr">
+        <is>
+          <t>Arrow of Light</t>
+        </is>
+      </c>
+      <c r="B81" s="13" t="inlineStr">
+        <is>
+          <t>February 2027</t>
+        </is>
+      </c>
+      <c r="C81" s="13" t="inlineStr">
+        <is>
+          <t>Citizenship &amp; Duty to God</t>
+        </is>
+      </c>
+      <c r="D81" s="13" t="inlineStr">
+        <is>
+          <t>Thu Feb 11</t>
+        </is>
+      </c>
+      <c r="E81" s="13" t="inlineStr">
+        <is>
+          <t>Duty to God: Reverence &amp; Service</t>
+        </is>
+      </c>
+      <c r="F81" s="13" t="inlineStr">
+        <is>
+          <t>Duty to God 2 (Meet a representative of a faith-based organization that assists people in crisis regardless of faith - guest or visit)
+Duty to God 1 &amp; 3 wrap-up (family faith/value discussion and daily-practice discussion - completed with parent/guardian or adult leader)</t>
+        </is>
+      </c>
+      <c r="G81" s="13" t="inlineStr">
+        <is>
+          <t>index cards, pencils, guest/visit confirmation, thank-you card, question cards</t>
+        </is>
+      </c>
+      <c r="H81" s="13" t="inlineStr">
+        <is>
+          <t>Finish the family faith/value discussion (req 1) and the daily-practice discussion (req 3) at home if not done.
+This is the LAST required adventure - confirm all six are recorded in Scoutbook so the Scout is ready to cross over.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="14" t="inlineStr">
+        <is>
+          <t>Arrow of Light</t>
+        </is>
+      </c>
+      <c r="B82" s="13" t="inlineStr">
+        <is>
+          <t>March 2027</t>
+        </is>
+      </c>
+      <c r="C82" s="13" t="inlineStr">
+        <is>
+          <t>Complete - Optional: Knife Safety</t>
+        </is>
+      </c>
+      <c r="D82" s="13" t="inlineStr">
+        <is>
+          <t>Thu Mar 4</t>
+        </is>
+      </c>
+      <c r="E82" s="13" t="inlineStr">
+        <is>
+          <t>Knife Rules and Safety Circle (optional)</t>
+        </is>
+      </c>
+      <c r="F82" s="13" t="inlineStr">
+        <is>
+          <t>Optional elective - Knife Safety 1 (Rules and promise)
+Knife Safety 2 (Safety circle)
+Knife Safety 3 (Care for and use a knife safely)</t>
+        </is>
+      </c>
       <c r="G82" s="13" t="inlineStr">
         <is>
-          <t>packing checklist, pencils, sample gear, BSA SAFE Checklist, chart paper, markers, camp map, printed site map or blank paper</t>
+          <t>printed Cub Scout Knife Safety Rules, pencils, trainer knives or approved pocketknives, work gloves if desired, clean cloth, small sharpening stone for demo only</t>
         </is>
       </c>
       <c r="H82" s="13" t="inlineStr">
         <is>
-          <t>Pack for the March 5-7 spring campout using tonight's checklist.
-Bring weather layers, sleeping gear, water bottle, and any required forms.</t>
+          <t>Tell families whether Scouts may bring an approved pocketknife next time and what supervision rules apply.
+This is enrichment - it also front-loads the Scouts BSA Totin' Chip.</t>
         </is>
       </c>
     </row>
@@ -4716,7 +4722,7 @@
       </c>
       <c r="C83" s="13" t="inlineStr">
         <is>
-          <t>Outdoor Adventurer</t>
+          <t>Complete - Optional: Knife Safety</t>
         </is>
       </c>
       <c r="D83" s="13" t="inlineStr">
@@ -4726,25 +4732,24 @@
       </c>
       <c r="E83" s="13" t="inlineStr">
         <is>
-          <t>Campout Debrief and Outdoor Ethics</t>
+          <t>Whittle a Useful Object (optional)</t>
         </is>
       </c>
       <c r="F83" s="13" t="inlineStr">
         <is>
-          <t>Outdoor Adventurer 5 (Participated in campout - outing)
-Outdoor Adventurer 6 (Campsite setup and patrol gear - outing)
-Outdoor Adventurer 7 (Food safety/kitchen sanitation - outing)
-Outdoor Adventurer 8 (Discuss what went well/differently; Outdoor Code and Leave No Trace Principles for Kids)</t>
+          <t>Optional elective - Knife Safety 4 (Make a useful object)
+Knife Safety 5 (Correct cooking knife; slice, chop, mince)</t>
         </is>
       </c>
       <c r="G83" s="13" t="inlineStr">
         <is>
-          <t>chart paper, markers, service/campout attendance notes, Outdoor Code card, Leave No Trace Principles for Kids cards</t>
+          <t>approved pocketknives, soft wood blanks or sticks, cut-resistant gloves if available, drop cloth, first-aid kit, cutting boards, paring knife, chef's knife, serrated knife, soft foods such as bananas, cucumbers, or herbs, sanitizer and paper towels</t>
         </is>
       </c>
       <c r="H83" s="13" t="inlineStr">
         <is>
-          <t>Air out and store gear. Thank the adult who helped you get to the campout.</t>
+          <t>Keep practicing safe knife habits in your new Scouts BSA troop.
+Ask your troop about earning the Totin' Chip.</t>
         </is>
       </c>
     </row>
@@ -4761,7 +4766,7 @@
       </c>
       <c r="C84" s="13" t="inlineStr">
         <is>
-          <t>Knife Safety (elective) + Catch-Up</t>
+          <t>Crossed Over - Mentor &amp; Celebrate</t>
         </is>
       </c>
       <c r="D84" s="13" t="inlineStr">
@@ -4771,25 +4776,23 @@
       </c>
       <c r="E84" s="13" t="inlineStr">
         <is>
-          <t>Knife Rules and Safety Circle</t>
+          <t>Mentor a Younger Den (optional)</t>
         </is>
       </c>
       <c r="F84" s="13" t="inlineStr">
         <is>
-          <t>Knife Safety 1 (Read, understand, and promise to follow Cub Scout Knife Safety Rules)
-Knife Safety 2 (Demonstrate knife safety circle)
-Knife Safety 3 (Care for and use a knife safely)</t>
+          <t>No required adventure - leadership/service bonus</t>
         </is>
       </c>
       <c r="G84" s="13" t="inlineStr">
         <is>
-          <t>printed Cub Scout Knife Safety Rules, pencils, trainer knives or approved pocketknives, work gloves if desired, clean cloth, small sharpening stone for demo only</t>
+          <t>chosen station supplies</t>
         </is>
       </c>
       <c r="H84" s="13" t="inlineStr">
         <is>
-          <t>Tell families whether Scouts may bring an approved pocketknife next time and what supervision rules apply.
-Check Scoutbook for any missing required-adventure items.</t>
+          <t>Keep showing up for your troop first; help the pack when you can.
+Invite your family to the April 29 End-of-Year Awards.</t>
         </is>
       </c>
     </row>
@@ -4806,7 +4809,7 @@
       </c>
       <c r="C85" s="13" t="inlineStr">
         <is>
-          <t>Knife Safety (elective) + Catch-Up</t>
+          <t>Crossed Over - Mentor &amp; Celebrate</t>
         </is>
       </c>
       <c r="D85" s="13" t="inlineStr">
@@ -4816,24 +4819,22 @@
       </c>
       <c r="E85" s="13" t="inlineStr">
         <is>
-          <t>Whittle a Useful Object and Kitchen Cuts</t>
+          <t>End-of-Year Send-Off (optional)</t>
         </is>
       </c>
       <c r="F85" s="13" t="inlineStr">
         <is>
-          <t>Knife Safety 4 (Use a pocketknife to make a useful object)
-Knife Safety 5 (Choose correct cooking knife and demonstrate slice, chop, mince)</t>
+          <t>No required adventure - celebration</t>
         </is>
       </c>
       <c r="G85" s="13" t="inlineStr">
         <is>
-          <t>approved pocketknives, soft wood blanks or sticks, cut-resistant gloves if available, drop cloth, first-aid kit, cutting boards, paring knife, chef's knife, serrated knife, soft foods such as bananas, cucumbers, or herbs, sanitizer and paper towels</t>
+          <t>awards/certificates from the pack, campfire program</t>
         </is>
       </c>
       <c r="H85" s="13" t="inlineStr">
         <is>
-          <t>Bring any final make-up evidence before the April 29 End-of-Year Awards and crossover.
-Celebrate crossing over - keep practicing safe knife habits in Scouts BSA.</t>
+          <t>Congratulations - you finished Cub Scouting and crossed over! Be Prepared and Do a Good Turn Daily.</t>
         </is>
       </c>
     </row>
@@ -5138,27 +5139,27 @@
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
+          <t>[ ] Outdoor Adventurer</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
           <t>[ ] Personal Fitness</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
-        <is>
-          <t>[ ] Citizenship</t>
-        </is>
-      </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>[ ] Duty to God</t>
+          <t>[ ] Citizenship &amp; Duty to God</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>[ ] Outdoor Adventurer</t>
+          <t>[ ] Complete - Optional: Knife Safety</t>
         </is>
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>[ ] Knife Safety (elective) + Catch-Up</t>
+          <t>[ ] Crossed Over - Mentor &amp; Celebrate</t>
         </is>
       </c>
     </row>

</xml_diff>